<commit_message>
Working cbuildv1p0 and acceleration testing results
Tested different TC settings and their impact on acceleration times.
</commit_message>
<xml_diff>
--- a/Control Algorithms/V1/CarSim Builds/V1.0 Signals and Variables List.xlsx
+++ b/Control Algorithms/V1/CarSim Builds/V1.0 Signals and Variables List.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GITHUB\FB26_Controls\Control Algorithms\V1\Architecture\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GITHUB\FB26_Controls\Control Algorithms\V1\CarSim Builds\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22FB7B9E-9E1E-4B73-8542-E789B705DCB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4684B0F-1BB5-4035-84B9-6948A66EEA49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-90" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{369501CE-6CA8-45C0-AE74-A62BF0386ED2}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="96">
   <si>
     <t>Signal</t>
   </si>
@@ -316,6 +316,15 @@
   </si>
   <si>
     <t>The percent of power the traction control cuts by</t>
+  </si>
+  <si>
+    <t>RPM to Radians per Second Conversion</t>
+  </si>
+  <si>
+    <t>rpm_to_radpers</t>
+  </si>
+  <si>
+    <t>(rad/s)/rpm</t>
   </si>
 </sst>
 </file>
@@ -1028,12 +1037,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E40D3DF-DFC2-4EE4-8BC8-226388D2D6FF}">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="34.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="36" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="22.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.42578125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="105.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1061,8 +1071,8 @@
       <c r="B2" t="s">
         <v>36</v>
       </c>
-      <c r="C2" t="s">
-        <v>10</v>
+      <c r="C2">
+        <v>1</v>
       </c>
       <c r="D2" t="s">
         <v>37</v>
@@ -1078,8 +1088,9 @@
       <c r="B3" t="s">
         <v>44</v>
       </c>
-      <c r="C3" t="s">
-        <v>10</v>
+      <c r="C3">
+        <f>1/9</f>
+        <v>0.1111111111111111</v>
       </c>
       <c r="D3" t="s">
         <v>45</v>
@@ -1160,11 +1171,28 @@
       <c r="B8" t="s">
         <v>91</v>
       </c>
+      <c r="C8">
+        <v>0.5</v>
+      </c>
       <c r="D8" t="s">
         <v>10</v>
       </c>
       <c r="E8" t="s">
         <v>92</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>93</v>
+      </c>
+      <c r="B9" t="s">
+        <v>94</v>
+      </c>
+      <c r="C9">
+        <v>0.10471999999999999</v>
+      </c>
+      <c r="D9" t="s">
+        <v>95</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
V1 variable list updated
</commit_message>
<xml_diff>
--- a/Control Algorithms/V1/CarSim Builds/V1.0 Signals and Variables List.xlsx
+++ b/Control Algorithms/V1/CarSim Builds/V1.0 Signals and Variables List.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GITHUB\FB26_Controls\Control Algorithms\V1\CarSim Builds\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4684B0F-1BB5-4035-84B9-6948A66EEA49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C204AA0-B4D7-4844-862A-433801211100}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-90" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{369501CE-6CA8-45C0-AE74-A62BF0386ED2}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="154">
   <si>
     <t>Signal</t>
   </si>
@@ -315,9 +315,6 @@
     <t>TC_CUT</t>
   </si>
   <si>
-    <t>The percent of power the traction control cuts by</t>
-  </si>
-  <si>
     <t>RPM to Radians per Second Conversion</t>
   </si>
   <si>
@@ -325,6 +322,183 @@
   </si>
   <si>
     <t>(rad/s)/rpm</t>
+  </si>
+  <si>
+    <t>m/s to kph Conversion</t>
+  </si>
+  <si>
+    <t>mpersec_to_kph</t>
+  </si>
+  <si>
+    <t>m/s / kph</t>
+  </si>
+  <si>
+    <t>Pack Enthalpy</t>
+  </si>
+  <si>
+    <t>h_pack</t>
+  </si>
+  <si>
+    <t>Busbar Enthalpy</t>
+  </si>
+  <si>
+    <t>h_busbar</t>
+  </si>
+  <si>
+    <t>J/kg</t>
+  </si>
+  <si>
+    <t>Gravitational Constant</t>
+  </si>
+  <si>
+    <t>g</t>
+  </si>
+  <si>
+    <t>m/s^2</t>
+  </si>
+  <si>
+    <t>Guestimate value</t>
+  </si>
+  <si>
+    <t>Battery Cell Mass</t>
+  </si>
+  <si>
+    <t>cell_mass</t>
+  </si>
+  <si>
+    <t>kg</t>
+  </si>
+  <si>
+    <t>Battery Cell Heat Capacity</t>
+  </si>
+  <si>
+    <t>cell_cp</t>
+  </si>
+  <si>
+    <t>J/kg*k</t>
+  </si>
+  <si>
+    <t>Off of the internet</t>
+  </si>
+  <si>
+    <t>Busbar Thermal Contact Resistance</t>
+  </si>
+  <si>
+    <t>busbar_thermalcontact_resistance</t>
+  </si>
+  <si>
+    <t>ohms</t>
+  </si>
+  <si>
+    <t>The resistance between the busbar and the contacts on the module</t>
+  </si>
+  <si>
+    <t>Busbar Resistivity</t>
+  </si>
+  <si>
+    <t>busbar_resistivity</t>
+  </si>
+  <si>
+    <t>ohm meters</t>
+  </si>
+  <si>
+    <t>Busbar Mass</t>
+  </si>
+  <si>
+    <t>busbar_mass</t>
+  </si>
+  <si>
+    <t>Busbar Length</t>
+  </si>
+  <si>
+    <t>busbar_length</t>
+  </si>
+  <si>
+    <t>Busbar Heat Capacity</t>
+  </si>
+  <si>
+    <t>busbar_Cp</t>
+  </si>
+  <si>
+    <t>Aluminums heat capacity from the internet</t>
+  </si>
+  <si>
+    <t>Busbar Cross Sectional Area</t>
+  </si>
+  <si>
+    <t>busbar_CC_area</t>
+  </si>
+  <si>
+    <t>m^2</t>
+  </si>
+  <si>
+    <t>Ambient Air Temperature</t>
+  </si>
+  <si>
+    <t>T_amb</t>
+  </si>
+  <si>
+    <t xml:space="preserve">k </t>
+  </si>
+  <si>
+    <t>24 degrees C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">100 minus the percent of power the traction control cuts by </t>
+  </si>
+  <si>
+    <t>SoC_initial</t>
+  </si>
+  <si>
+    <t>Initial State of Charge</t>
+  </si>
+  <si>
+    <t>Cells in Series</t>
+  </si>
+  <si>
+    <t>S</t>
+  </si>
+  <si>
+    <t>The number of cells in series inside of the battery pack</t>
+  </si>
+  <si>
+    <t>Maximum Current</t>
+  </si>
+  <si>
+    <t>I_max</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>Gear Ratio</t>
+  </si>
+  <si>
+    <t>GR</t>
+  </si>
+  <si>
+    <t>Nominal Cell Capacity</t>
+  </si>
+  <si>
+    <t>C_nominal</t>
+  </si>
+  <si>
+    <t>Ah</t>
+  </si>
+  <si>
+    <t>A_pack</t>
+  </si>
+  <si>
+    <t>Battery Pack Surface Area</t>
+  </si>
+  <si>
+    <t>The  surface area of the outside of the pack casing</t>
+  </si>
+  <si>
+    <t>Busbar Surface Area</t>
+  </si>
+  <si>
+    <t>A_busbar</t>
   </si>
 </sst>
 </file>
@@ -368,9 +542,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1037,7 +1212,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E40D3DF-DFC2-4EE4-8BC8-226388D2D6FF}">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="36" bestFit="1" customWidth="1"/>
@@ -1178,21 +1353,325 @@
         <v>10</v>
       </c>
       <c r="E8" t="s">
-        <v>92</v>
+        <v>135</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>92</v>
+      </c>
+      <c r="B9" t="s">
         <v>93</v>
-      </c>
-      <c r="B9" t="s">
-        <v>94</v>
       </c>
       <c r="C9">
         <v>0.10471999999999999</v>
       </c>
       <c r="D9" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
         <v>95</v>
+      </c>
+      <c r="B10" t="s">
+        <v>96</v>
+      </c>
+      <c r="C10">
+        <v>3.6</v>
+      </c>
+      <c r="D10" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>98</v>
+      </c>
+      <c r="B11" t="s">
+        <v>99</v>
+      </c>
+      <c r="C11">
+        <v>5</v>
+      </c>
+      <c r="D11" t="s">
+        <v>102</v>
+      </c>
+      <c r="E11" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>100</v>
+      </c>
+      <c r="B12" t="s">
+        <v>101</v>
+      </c>
+      <c r="C12">
+        <v>5</v>
+      </c>
+      <c r="D12" t="s">
+        <v>102</v>
+      </c>
+      <c r="E12" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>103</v>
+      </c>
+      <c r="B13" t="s">
+        <v>104</v>
+      </c>
+      <c r="C13">
+        <v>9.8000000000000007</v>
+      </c>
+      <c r="D13" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>107</v>
+      </c>
+      <c r="B14" t="s">
+        <v>108</v>
+      </c>
+      <c r="C14">
+        <v>4.5999999999999999E-2</v>
+      </c>
+      <c r="D14" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>110</v>
+      </c>
+      <c r="B15" t="s">
+        <v>111</v>
+      </c>
+      <c r="C15">
+        <v>1000</v>
+      </c>
+      <c r="D15" t="s">
+        <v>112</v>
+      </c>
+      <c r="E15" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>114</v>
+      </c>
+      <c r="B16" t="s">
+        <v>115</v>
+      </c>
+      <c r="C16" s="2">
+        <v>1.6800000000000002E-8</v>
+      </c>
+      <c r="D16" t="s">
+        <v>116</v>
+      </c>
+      <c r="E16" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>118</v>
+      </c>
+      <c r="B17" t="s">
+        <v>119</v>
+      </c>
+      <c r="C17" s="2">
+        <v>1.6800000000000002E-8</v>
+      </c>
+      <c r="D17" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>121</v>
+      </c>
+      <c r="B18" t="s">
+        <v>122</v>
+      </c>
+      <c r="C18">
+        <v>0.01</v>
+      </c>
+      <c r="D18" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>123</v>
+      </c>
+      <c r="B19" t="s">
+        <v>124</v>
+      </c>
+      <c r="C19">
+        <v>3.2000000000000001E-2</v>
+      </c>
+      <c r="D19" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>125</v>
+      </c>
+      <c r="B20" t="s">
+        <v>126</v>
+      </c>
+      <c r="C20">
+        <v>237</v>
+      </c>
+      <c r="D20" t="s">
+        <v>112</v>
+      </c>
+      <c r="E20" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>128</v>
+      </c>
+      <c r="B21" t="s">
+        <v>129</v>
+      </c>
+      <c r="C21">
+        <v>1.08E-4</v>
+      </c>
+      <c r="D21" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>131</v>
+      </c>
+      <c r="B22" t="s">
+        <v>132</v>
+      </c>
+      <c r="C22">
+        <v>297.14999999999998</v>
+      </c>
+      <c r="D22" t="s">
+        <v>133</v>
+      </c>
+      <c r="E22" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>137</v>
+      </c>
+      <c r="B23" t="s">
+        <v>136</v>
+      </c>
+      <c r="C23">
+        <v>1</v>
+      </c>
+      <c r="D23" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>138</v>
+      </c>
+      <c r="B24" t="s">
+        <v>139</v>
+      </c>
+      <c r="C24">
+        <v>138</v>
+      </c>
+      <c r="D24" t="s">
+        <v>10</v>
+      </c>
+      <c r="E24" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>141</v>
+      </c>
+      <c r="B25" t="s">
+        <v>142</v>
+      </c>
+      <c r="C25">
+        <v>157.69999999999999</v>
+      </c>
+      <c r="D25" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>144</v>
+      </c>
+      <c r="B26" t="s">
+        <v>145</v>
+      </c>
+      <c r="C26">
+        <v>14.14</v>
+      </c>
+      <c r="D26" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>146</v>
+      </c>
+      <c r="B27" t="s">
+        <v>147</v>
+      </c>
+      <c r="C27">
+        <v>3</v>
+      </c>
+      <c r="D27" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>150</v>
+      </c>
+      <c r="B28" t="s">
+        <v>149</v>
+      </c>
+      <c r="C28">
+        <v>0.71162624799999996</v>
+      </c>
+      <c r="D28" t="s">
+        <v>130</v>
+      </c>
+      <c r="E28" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>152</v>
+      </c>
+      <c r="B29" t="s">
+        <v>153</v>
+      </c>
+      <c r="C29">
+        <v>1.5E-3</v>
+      </c>
+      <c r="D29" t="s">
+        <v>130</v>
       </c>
     </row>
   </sheetData>

</xml_diff>